<commit_message>
v0.4: SoT-based input sheet skeleton (DTO/Request/Blade/Controller/Test)
</commit_message>
<xml_diff>
--- a/tests/Fixtures/個人住民税vol23.xlsx
+++ b/tests/Fixtures/個人住民税vol23.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4245ae31b7bca767/Desktop/ふるさと納税クラウド/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{823BF139-23A2-4907-AC15-57EEEB3CEE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{E8F1E613-22D3-4668-A0D3-EEF16E5E6BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A72DF1B8-8E30-497E-A581-282B3B8A1B07}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12672" yWindow="756" windowWidth="16128" windowHeight="15432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="インプット表" sheetId="1" r:id="rId1"/>
@@ -250,7 +250,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="287">
   <si>
     <t>前期</t>
   </si>
@@ -1559,14 +1559,6 @@
   </si>
   <si>
     <t>ワンストップ適用フラグ</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>寄付先団体数</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>所得税申告</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
@@ -3172,6 +3164,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
   <a:themeElements>
@@ -3526,7 +3522,7 @@
         <v>12202436</v>
       </c>
       <c r="D2" s="12">
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="H2" t="s">
         <v>2</v>
@@ -3535,7 +3531,7 @@
         <v>703890</v>
       </c>
       <c r="K2" s="12">
-        <v>630000</v>
+        <v>327927</v>
       </c>
       <c r="P2" s="6"/>
       <c r="Q2" t="s">
@@ -3728,13 +3724,13 @@
         <v>18</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="K18" s="3">
         <v>1000000</v>
       </c>
       <c r="M18" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
@@ -3784,7 +3780,7 @@
         <v>448000</v>
       </c>
       <c r="K22" s="12">
-        <v>48000</v>
+        <v>464000</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
@@ -3833,7 +3829,7 @@
       </c>
       <c r="K30" s="3">
         <f>SUM(K22,K27,K28)</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
@@ -3846,7 +3842,7 @@
       </c>
       <c r="K31" s="3">
         <f>K22</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
     </row>
     <row r="33" spans="8:11" x14ac:dyDescent="0.45">
@@ -3854,33 +3850,17 @@
         <v>175</v>
       </c>
       <c r="J33" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="K33" s="3" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="34" spans="8:11" x14ac:dyDescent="0.45">
-      <c r="H34" t="s">
-        <v>176</v>
-      </c>
-      <c r="J34" s="3">
-        <v>10</v>
-      </c>
-      <c r="K34" s="3">
-        <v>1</v>
-      </c>
+      <c r="H34"/>
     </row>
     <row r="35" spans="8:11" x14ac:dyDescent="0.45">
-      <c r="H35" t="s">
-        <v>177</v>
-      </c>
-      <c r="J35" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K35" s="3" t="b">
-        <v>0</v>
-      </c>
+      <c r="H35"/>
     </row>
     <row r="37" spans="8:11" x14ac:dyDescent="0.45">
       <c r="H37" s="2" t="s">
@@ -4005,11 +3985,11 @@
       </c>
       <c r="P6" s="3">
         <f>SUM(J40:J43)</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="Q6" s="3">
         <f>SUM(J40:J43)</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="T6" t="s">
         <v>43</v>
@@ -4032,14 +4012,14 @@
       </c>
       <c r="AB6" s="3">
         <f>SUM(P6,P38,P39)</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="AD6" s="3" t="s">
         <v>56</v>
       </c>
       <c r="AE6" s="3">
         <f>Q67-P67</f>
-        <v>7760</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="3"/>
     </row>
@@ -4060,7 +4040,7 @@
         <v>111</v>
       </c>
       <c r="T7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V7" s="3">
         <f>IF(ROUNDDOWN(AA6-AA24,-3)&lt;0,0,ROUNDDOWN(AA6-AA24,-3))</f>
@@ -4068,11 +4048,11 @@
       </c>
       <c r="W7" s="3">
         <f>IF(ROUNDDOWN(AB6-AB24,-3)&lt;0,0,ROUNDDOWN(AB6-AB24,-3))</f>
-        <v>3530000</v>
+        <v>11882000</v>
       </c>
       <c r="X7" s="3">
         <f>IF(ROUNDDOWN(AB6-AB24,-3)&lt;0,0,ROUNDDOWN(AB6-AB24,-3))</f>
-        <v>3530000</v>
+        <v>11882000</v>
       </c>
       <c r="Z7"/>
       <c r="AD7" s="3" t="s">
@@ -4080,7 +4060,7 @@
       </c>
       <c r="AE7" s="3">
         <f>W38</f>
-        <v>41305</v>
+        <v>439002</v>
       </c>
       <c r="AF7" s="3"/>
     </row>
@@ -4143,14 +4123,14 @@
       </c>
       <c r="P8" s="3">
         <f>インプット表!K2</f>
-        <v>630000</v>
+        <v>327927</v>
       </c>
       <c r="Q8" s="3">
         <f>インプット表!K2</f>
-        <v>630000</v>
+        <v>327927</v>
       </c>
       <c r="T8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V8" s="3">
         <f>インプット表!J30</f>
@@ -4158,7 +4138,7 @@
       </c>
       <c r="W8" s="3">
         <f>インプット表!K30</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
       <c r="X8" s="3">
         <v>0</v>
@@ -4172,14 +4152,14 @@
       </c>
       <c r="AB8" s="3">
         <f t="shared" si="0"/>
-        <v>630000</v>
+        <v>327927</v>
       </c>
       <c r="AD8" s="3" t="s">
         <v>48</v>
       </c>
       <c r="AE8" s="3">
         <f>SUM(AE6:AE7)</f>
-        <v>49065</v>
+        <v>439002</v>
       </c>
       <c r="AF8" s="3"/>
       <c r="AG8" s="5"/>
@@ -4247,7 +4227,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="V9" s="3">
         <f>インプット表!J22</f>
@@ -4255,7 +4235,7 @@
       </c>
       <c r="W9" s="3">
         <f>インプット表!K22</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
       <c r="X9" s="3">
         <v>0</v>
@@ -4331,7 +4311,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="Z10" t="s">
         <v>9</v>
@@ -4396,7 +4376,7 @@
   +P37*IF(W6=TRUE,マスター!$L$15,マスター!$N$15)
   +P38*IF(W6=TRUE,マスター!$L$16,マスター!$N$16)
   +P39*IF(W6=TRUE,マスター!$L$17,マスター!$N$17)</f>
-        <v>211800</v>
+        <v>712920</v>
       </c>
       <c r="X11" s="3">
         <f>X7*IF(X6=TRUE,マスター!$L$4,マスター!$N$4)
@@ -4413,7 +4393,7 @@
   +Q37*IF(X6=TRUE,マスター!$L$15,マスター!$N$15)
   +Q38*IF(X6=TRUE,マスター!$L$16,マスター!$N$16)
   +Q39*IF(X6=TRUE,マスター!$L$17,マスター!$N$17)</f>
-        <v>211800</v>
+        <v>712920</v>
       </c>
       <c r="Z11" t="s">
         <v>12</v>
@@ -4493,7 +4473,7 @@
   +P37*IF(W6=TRUE,マスター!$M$15,マスター!$O$15)
   +P38*IF(W6=TRUE,マスター!$M$16,マスター!$O$16)
   +P39*IF(W6=TRUE,マスター!$M$17,マスター!$O$17)</f>
-        <v>141200</v>
+        <v>475280</v>
       </c>
       <c r="X12" s="3">
         <f>X7*IF(X6=TRUE,マスター!$M$4,マスター!$O$4)
@@ -4510,7 +4490,7 @@
   +Q37*IF(X6=TRUE,マスター!$M$15,マスター!$O$15)
   +Q38*IF(X6=TRUE,マスター!$M$16,マスター!$O$16)
   +Q39*IF(X6=TRUE,マスター!$M$17,マスター!$O$17)</f>
-        <v>141200</v>
+        <v>475280</v>
       </c>
       <c r="Z12" t="s">
         <v>14</v>
@@ -4615,7 +4595,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Z13" t="s">
         <v>17</v>
@@ -4959,7 +4939,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="Z16" t="s">
         <v>29</v>
@@ -5118,14 +5098,14 @@
       </c>
       <c r="W17" s="3">
         <f t="shared" ref="W17:X18" si="3">W11-W14</f>
-        <v>210300</v>
+        <v>711420</v>
       </c>
       <c r="X17" s="3">
         <f t="shared" si="3"/>
-        <v>210300</v>
+        <v>711420</v>
       </c>
       <c r="Z17" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AA17" s="3" cm="1">
         <f t="array" ref="AA17">IF(
@@ -5230,11 +5210,11 @@
       </c>
       <c r="W18" s="3">
         <f>W12-W15</f>
-        <v>140200</v>
+        <v>474280</v>
       </c>
       <c r="X18" s="3">
         <f t="shared" si="3"/>
-        <v>140200</v>
+        <v>474280</v>
       </c>
       <c r="Z18" t="s">
         <v>33</v>
@@ -5257,7 +5237,7 @@
         <v>13831070</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="O19" s="3" cm="1">
         <f t="array" ref="O19">IF(O6=0,0,INDEX({0,630000,610000,510000,410000,310000,210000,110000,60000,30000,0},
@@ -5283,18 +5263,16 @@
       </c>
       <c r="W19" s="3">
         <f>SUM(W17:W18)</f>
-        <v>350500</v>
+        <v>1185700</v>
       </c>
       <c r="X19" s="3">
         <f>SUM(X17:X18)</f>
-        <v>350500</v>
+        <v>1185700</v>
       </c>
       <c r="Z19" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="AA19" s="3" cm="1">
-        <f t="array" ref="AA19">IF(AA6=0,0,INDEX({0,630000,610000,510000,410000,310000,210000,110000,60000,30000,0},
-MATCH(_xlfn.NUMBERVALUE(インプット表!J18),{0,580001,850001,900001,950001,1000001,1050001,1100001,1150001,1200001,1230001},1)))</f>
+        <v>285</v>
+      </c>
+      <c r="AA19" s="3">
         <v>0</v>
       </c>
       <c r="AB19" s="3" cm="1">
@@ -5308,25 +5286,25 @@
         <v>49</v>
       </c>
       <c r="O20" s="3" cm="1">
-        <f t="array" ref="O20">IF(O6=0,0,INDEX({950000,880000,680000,630000,580000,480000,320000,160000,0},
-MATCH(_xlfn.NUMBERVALUE(SUM(O6,O29:O39)),{0,1320001,3360001,4890001,6550001,23500001,24000001,24500001,25000001},1)))</f>
-        <v>580000</v>
+        <f t="array" ref="O20">IF(O6=0,0,INDEX({480000,320000,160000,0},
+MATCH(_xlfn.NUMBERVALUE(SUM(O6,O29:O39)),{0,24000001,24500001,25000001},1)))</f>
+        <v>480000</v>
       </c>
       <c r="P20" s="3" cm="1">
         <f t="array" ref="P20">IF(P6=0,0,INDEX({950000,880000,680000,630000,580000,480000,320000,160000,0},
 MATCH(_xlfn.NUMBERVALUE(SUM(P6,P29:P39)),{0,1320001,3360001,4890001,6550001,23500001,24000001,24500001,25000001},1)))</f>
-        <v>630000</v>
+        <v>580000</v>
       </c>
       <c r="Q20" s="3" cm="1">
         <f t="array" ref="Q20">IF(Q6=0,0,INDEX({950000,880000,680000,630000,580000,480000,320000,160000,0},
 MATCH(_xlfn.NUMBERVALUE(SUM(Q6,Q29:Q39)),{0,1320001,3360001,4890001,6550001,23500001,24000001,24500001,25000001},1)))</f>
-        <v>630000</v>
+        <v>580000</v>
       </c>
       <c r="T20" t="s">
         <v>50</v>
       </c>
       <c r="Z20" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AA20" s="3" cm="1">
         <f t="array" ref="AA20">INDEX({430000,290000,150000,0},
@@ -5391,15 +5369,15 @@
       </c>
       <c r="O21" s="3">
         <f>SUM(O8:O20)</f>
-        <v>1283890</v>
+        <v>1183890</v>
       </c>
       <c r="P21" s="3">
         <f>SUM(P8:P20)</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="Q21" s="3">
         <f>SUM(Q8:Q20)</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="U21" t="s">
         <v>45</v>
@@ -5414,7 +5392,7 @@
         <f>IF(N(インプット表!$K$30)&lt;=2000,0,
       (MIN(N(インプット表!$K$30), SUM(Q42:Q48)*0.3)-2000)
       *IF($W$6=TRUE, マスター!$L$19, マスター!$N$19))</f>
-        <v>2760</v>
+        <v>27720</v>
       </c>
       <c r="X21" s="12">
         <f xml:space="preserve"> IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
@@ -5508,7 +5486,7 @@
         <f>IF(N(インプット表!$K$30)&lt;=2000,0,
        (MIN(N(インプット表!$K$30), SUM(Q42:Q48)*0.3)-2000)
        *IF($W$6=TRUE, マスター!$M$19, マスター!$O$19))</f>
-        <v>1840</v>
+        <v>18480</v>
       </c>
       <c r="X22" s="12">
         <f xml:space="preserve"> IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
@@ -5668,7 +5646,7 @@
       </c>
       <c r="P24" s="3">
         <f>IF(W32,0,IF(インプット表!K21+インプット表!K22&lt;2000,0,IF(インプット表!K21&lt;=SUM(P6,P29:P39)*0.4,インプット表!K21,SUM(P6,P29:P39)*0.4)+インプット表!K22-2000))</f>
-        <v>46000</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="12">
         <v>0</v>
@@ -5688,7 +5666,7 @@
 IF(N(インプット表!$K$31)&lt;=2000, 0,
    (N(インプット表!$K$31)-2000) * $AB$56 * IF($W$6, マスター!$L$20, マスター!$N$20)
 )</f>
-        <v>22022.04</v>
+        <v>156083.00399999999</v>
       </c>
       <c r="X24" s="12">
         <v>0</v>
@@ -5702,7 +5680,7 @@
       </c>
       <c r="AB24" s="3">
         <f>SUM(AB8:AB23)</f>
-        <v>1470000</v>
+        <v>1167927</v>
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.45">
@@ -5766,15 +5744,15 @@
       </c>
       <c r="O25" s="3">
         <f>SUM(O21:O24)</f>
-        <v>1876927</v>
+        <v>1776927</v>
       </c>
       <c r="P25" s="3">
         <f>SUM(P21:P24)</f>
-        <v>1716000</v>
+        <v>1317927</v>
       </c>
       <c r="Q25" s="3">
         <f>SUM(Q21:Q24)</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="U25" t="s">
         <v>46</v>
@@ -5791,7 +5769,7 @@
 IF(N(インプット表!$K$31)&lt;=2000, 0,
    (N(インプット表!$K$31)-2000) * $AB$56 * IF($W$6, マスター!$M$20, マスター!$O$20)
 )</f>
-        <v>14681.36</v>
+        <v>104055.336</v>
       </c>
       <c r="X25" s="12">
         <v>0</v>
@@ -5837,7 +5815,7 @@
       </c>
       <c r="W27" s="3">
         <f>N($W$17)*0.2</f>
-        <v>42060</v>
+        <v>142284</v>
       </c>
       <c r="X27" s="12">
         <v>0</v>
@@ -5878,7 +5856,7 @@
       </c>
       <c r="W28" s="3">
         <f>N($W$18)*0.2</f>
-        <v>28040</v>
+        <v>94856</v>
       </c>
       <c r="X28" s="12">
         <v>0</v>
@@ -5938,7 +5916,7 @@
       </c>
       <c r="W30" s="3">
         <f>ROUNDUP(MIN(N($W$24), N($W$27)),0)</f>
-        <v>22023</v>
+        <v>142284</v>
       </c>
       <c r="X30" s="12">
         <v>0</v>
@@ -5984,7 +5962,7 @@
       </c>
       <c r="W31" s="3">
         <f>ROUNDUP(MIN(N($W$25),N($W$28)),0)</f>
-        <v>14682</v>
+        <v>94856</v>
       </c>
       <c r="X31" s="12">
         <v>0</v>
@@ -5993,11 +5971,11 @@
         <v>14</v>
       </c>
       <c r="AA31" s="3">
-        <f>O12-AA12</f>
+        <f t="shared" ref="AA31:AB37" si="4">O12-AA12</f>
         <v>0</v>
       </c>
       <c r="AB31" s="3">
-        <f>P12-AB12</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6018,29 +5996,29 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="V32" s="3" t="b">
-        <f xml:space="preserve"> AND( インプット表!$J$33, インプット表!$J$34&lt;=5, NOT(インプット表!$J$35) )</f>
+        <f>インプット表!$J$33</f>
         <v>0</v>
       </c>
       <c r="W32" s="3" t="b">
-        <f xml:space="preserve"> AND( インプット表!$K$33, インプット表!$K$34&lt;=5, NOT(インプット表!$K$35) )</f>
-        <v>0</v>
+        <f>インプット表!$K$33</f>
+        <v>1</v>
       </c>
       <c r="X32" s="3" t="b">
-        <f xml:space="preserve"> AND( インプット表!$K$33, インプット表!$K$34&lt;=5, NOT(インプット表!$K$35) )</f>
-        <v>0</v>
+        <f>インプット表!$K$33</f>
+        <v>1</v>
       </c>
       <c r="Z32" t="s">
         <v>17</v>
       </c>
       <c r="AA32" s="3">
-        <f>O13-AA13</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB32" s="3">
-        <f>P13-AB13</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6065,7 +6043,7 @@
       </c>
       <c r="R33" s="5"/>
       <c r="U33" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="V33" s="5" cm="1">
         <f t="array" ref="V33" xml:space="preserve">
@@ -6084,7 +6062,7 @@
 MAX(0,N(インプット表!$K$31)-2000)*AB56*INDEX(マスター!$AA$4:$AA$8,MATCH(1,(計算結果!$AB$49&gt;=マスター!$X$4:$X$8)*(計算結果!$AB$49&lt;=IF(マスター!$Z$4:$Z$8="",1E+99,マスター!$Z$4:$Z$8)),0))*IF($W$6,4/5,3/5),
 0
 ),0)</f>
-        <v>0</v>
+        <v>93397</v>
       </c>
       <c r="X33" s="12">
         <v>0</v>
@@ -6093,11 +6071,11 @@
         <v>19</v>
       </c>
       <c r="AA33" s="3">
-        <f>O14-AA14</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB33" s="3">
-        <f>P14-AB14</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6134,7 +6112,7 @@
       </c>
       <c r="T34"/>
       <c r="U34" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="V34" s="5" cm="1">
         <f t="array" ref="V34" xml:space="preserve">
@@ -6154,7 +6132,7 @@
 N($W$18)*0.2),
 0
 ),0)</f>
-        <v>0</v>
+        <v>62265</v>
       </c>
       <c r="X34" s="12">
         <v>0</v>
@@ -6163,11 +6141,11 @@
         <v>47</v>
       </c>
       <c r="AA34" s="3">
-        <f>O15-AA15</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB34" s="3">
-        <f>P15-AB15</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6237,11 +6215,11 @@
         <v>29</v>
       </c>
       <c r="AA35" s="3">
-        <f>O16-AA16</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB35" s="3">
-        <f>P16-AB16</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6308,7 +6286,7 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="U36" t="s">
         <v>45</v>
@@ -6319,7 +6297,7 @@
       </c>
       <c r="W36" s="3">
         <f>ROUNDUP($W$21+$W$33+$W$30,0)</f>
-        <v>24783</v>
+        <v>263401</v>
       </c>
       <c r="X36" s="12">
         <f>ROUNDDOWN(X21+X33,-2)</f>
@@ -6329,11 +6307,11 @@
         <v>31</v>
       </c>
       <c r="AA36" s="3">
-        <f>O17-AA17</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB36" s="3">
-        <f>P17-AB17</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6404,7 +6382,7 @@
       </c>
       <c r="W37" s="3">
         <f>ROUNDUP($W$22+$W$34+$W$31,0)</f>
-        <v>16522</v>
+        <v>175601</v>
       </c>
       <c r="X37" s="12">
         <f>ROUNDDOWN(X22+X34,-2)</f>
@@ -6414,11 +6392,11 @@
         <v>33</v>
       </c>
       <c r="AA37" s="3">
-        <f>O18-AA18</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AB37" s="3">
-        <f>P18-AB18</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6447,7 +6425,7 @@
       </c>
       <c r="W38" s="3">
         <f>SUM(W36:W37)</f>
-        <v>41305</v>
+        <v>439002</v>
       </c>
       <c r="X38" s="12">
         <f>SUM(X36:X37)</f>
@@ -6514,7 +6492,7 @@
       </c>
       <c r="C40" s="3">
         <f>SUM(インプット表!D2,インプット表!D3,インプット表!D4,IF(インプット表!D5&lt;0,0,インプット表!D5),IF(インプット表!D6&lt;0,0,インプット表!D6),IF(インプット表!D7&lt;0,0,インプット表!D7),IF(インプット表!D8&lt;0,0,インプット表!D8),IF(インプット表!D9&lt;0,0,インプット表!D9))</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="D40" s="66" t="s">
         <v>113</v>
@@ -6538,7 +6516,7 @@
  _xlpm.use_from_it,MIN(MAX(0,_xlpm.it_after), _xlpm.econ_neg-_xlpm.use_from_st-_xlpm.use_from_lt),
  _xlpm.econ_after + _xlpm.use_from_st + _xlpm.use_from_lt + _xlpm.use_from_it
 )</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="F40" s="67" t="s">
         <v>114</v>
@@ -6561,7 +6539,7 @@
  _xlpm.econ_when_neg, _xlpm.econ - _xlpm.use_from_econ,
  IF(_xlpm.forest&gt;=0, _xlpm.econ_when_pos, _xlpm.econ_when_neg)
 )</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="H40" s="67" t="s">
         <v>115</v>
@@ -6577,11 +6555,11 @@
  _xlpm.use_for,MIN(_xlpm.ret_pos-_xlpm.use_lt-_xlpm.use_st-_xlpm.use_econ,_xlpm.neg_for),
  _xlpm.econ + _xlpm.use_econ
 )</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="J40" s="3">
         <f>I40</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="L40" t="s">
         <v>82</v>
@@ -6595,11 +6573,11 @@
       </c>
       <c r="P40" s="3">
         <f>P6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="Q40" s="3">
         <f>Q6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="T40"/>
     </row>
@@ -6660,7 +6638,7 @@
         <v>0</v>
       </c>
       <c r="J41" s="3">
-        <f t="shared" ref="J41:J45" si="4">I41</f>
+        <f t="shared" ref="J41:J45" si="5">I41</f>
         <v>0</v>
       </c>
       <c r="M41" s="2" t="s">
@@ -6668,19 +6646,19 @@
       </c>
       <c r="O41" s="3">
         <f>MIN(O25, O40)</f>
-        <v>1876927</v>
+        <v>1776927</v>
       </c>
       <c r="P41" s="3">
         <f>MIN(P25, P40)</f>
-        <v>1716000</v>
+        <v>1317927</v>
       </c>
       <c r="Q41" s="3">
         <f>Q25</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="T41"/>
       <c r="Z41" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AA41" t="s">
         <v>0</v>
@@ -6754,15 +6732,15 @@
       </c>
       <c r="O42" s="3">
         <f>ROUNDDOWN(O40 - O41,-3)</f>
-        <v>11954000</v>
+        <v>12054000</v>
       </c>
       <c r="P42" s="3">
         <f>ROUNDDOWN(P40 - P41,-3)</f>
-        <v>3284000</v>
+        <v>11732000</v>
       </c>
       <c r="Q42" s="3">
         <f>ROUNDDOWN(Q40 - Q41,-3)</f>
-        <v>3330000</v>
+        <v>11732000</v>
       </c>
       <c r="T42"/>
       <c r="Z42" t="s">
@@ -6770,11 +6748,11 @@
       </c>
       <c r="AA42" s="5">
         <f>INDEX($O:$O, MATCH("総合課税",$M:$M,0))</f>
-        <v>11954000</v>
+        <v>12054000</v>
       </c>
       <c r="AB42" s="5">
         <f>INDEX($P:$P, MATCH("総合課税",$M:$M,0))</f>
-        <v>3284000</v>
+        <v>11732000</v>
       </c>
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.45">
@@ -6916,7 +6894,7 @@
         <v>0</v>
       </c>
       <c r="J44" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M44" s="2" t="s">
@@ -6977,7 +6955,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M45" s="2" t="s">
@@ -7013,21 +6991,21 @@
       </c>
       <c r="J46" s="3">
         <f>SUM(J40:J45)</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>78</v>
       </c>
       <c r="O46" s="3">
-        <f t="shared" ref="O46:Q47" si="5">ROUNDDOWN(O36,-3)</f>
+        <f t="shared" ref="O46:Q47" si="6">ROUNDDOWN(O36,-3)</f>
         <v>0</v>
       </c>
       <c r="P46" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Q46" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z46" t="s">
@@ -7047,15 +7025,15 @@
         <v>79</v>
       </c>
       <c r="O47" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="P47" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Q47" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z47" t="s">
@@ -7210,11 +7188,11 @@
       </c>
       <c r="AA49" s="14">
         <f>AA42-$AA$39</f>
-        <v>11904000</v>
+        <v>12004000</v>
       </c>
       <c r="AB49" s="14">
         <f>AB42-$AB$39</f>
-        <v>3234000</v>
+        <v>11682000</v>
       </c>
     </row>
     <row r="50" spans="1:32" x14ac:dyDescent="0.45">
@@ -7285,15 +7263,15 @@
       </c>
       <c r="O50" s="3" cm="1">
         <f t="array" ref="O50">O42*INDEX(マスター!$D$3:$D$9,MATCH(1,(O42&gt;=マスター!$A$3:$A$9)*(O42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))-INDEX(マスター!$E$3:$E$9,MATCH(1,(O42&gt;=マスター!$A$3:$A$9)*(O42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</f>
-        <v>2408820</v>
+        <v>2441820</v>
       </c>
       <c r="P50" s="3" cm="1">
         <f t="array" ref="P50">P42*INDEX(マスター!$D$3:$D$9,MATCH(1,(P42&gt;=マスター!$A$3:$A$9)*(P42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))-INDEX(マスター!$E$3:$E$9,MATCH(1,(P42&gt;=マスター!$A$3:$A$9)*(P42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</f>
-        <v>230900</v>
+        <v>2335560</v>
       </c>
       <c r="Q50" s="3" cm="1">
         <f t="array" ref="Q50">Q42*INDEX(マスター!$D$3:$D$9,MATCH(1,(Q42&gt;=マスター!$A$3:$A$9)*(Q42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))-INDEX(マスター!$E$3:$E$9,MATCH(1,(Q42&gt;=マスター!$A$3:$A$9)*(Q42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</f>
-        <v>238500</v>
+        <v>2335560</v>
       </c>
       <c r="Z50" t="s">
         <v>156</v>
@@ -7304,7 +7282,7 @@
       </c>
       <c r="AB50">
         <f>LOOKUP($AB$49, マスター!$Q$4:$Q$10, マスター!$V$4:$V$10)</f>
-        <v>0.79790000000000005</v>
+        <v>0.56306999999999996</v>
       </c>
     </row>
     <row r="51" spans="1:32" x14ac:dyDescent="0.45">
@@ -7524,7 +7502,7 @@
         <v>0</v>
       </c>
       <c r="P54" s="3">
-        <f t="shared" ref="O54:P55" si="6">P46*15%</f>
+        <f t="shared" ref="O54:P55" si="7">P46*15%</f>
         <v>0</v>
       </c>
       <c r="Q54" s="3">
@@ -7564,11 +7542,11 @@
         <v>79</v>
       </c>
       <c r="O55" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="P55" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="Q55" s="3">
@@ -7636,7 +7614,7 @@
   IF($AB$54&lt;&gt;"", $AB$54, 1),
   IF($AB$55&lt;&gt;"", $AB$55, 1)
 )</f>
-        <v>0.79790000000000005</v>
+        <v>0.56306999999999996</v>
       </c>
     </row>
     <row r="57" spans="1:32" x14ac:dyDescent="0.45">
@@ -7658,19 +7636,19 @@
     </row>
     <row r="59" spans="1:32" x14ac:dyDescent="0.45">
       <c r="M59" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="O59" s="3">
         <f>ROUNDDOWN(SUM(O50:O57),0)</f>
-        <v>2408820</v>
+        <v>2441820</v>
       </c>
       <c r="P59" s="3">
         <f>ROUNDDOWN(SUM(P50:P57),0)</f>
-        <v>230900</v>
+        <v>2335560</v>
       </c>
       <c r="Q59" s="3">
         <f>ROUNDDOWN(SUM(Q50:Q57),0)</f>
-        <v>238500</v>
+        <v>2335560</v>
       </c>
     </row>
     <row r="60" spans="1:32" x14ac:dyDescent="0.45">
@@ -7837,19 +7815,19 @@
     </row>
     <row r="63" spans="1:32" x14ac:dyDescent="0.45">
       <c r="M63" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="O63" s="3">
         <f>O59-SUM(O60:O62)</f>
-        <v>2403620</v>
+        <v>2436620</v>
       </c>
       <c r="P63" s="3">
         <f>P59-SUM(P60:P62)</f>
-        <v>230900</v>
+        <v>2335560</v>
       </c>
       <c r="Q63" s="3">
         <f>Q59-SUM(Q60:Q62)</f>
-        <v>238500</v>
+        <v>2335560</v>
       </c>
     </row>
     <row r="64" spans="1:32" x14ac:dyDescent="0.45">
@@ -7875,15 +7853,15 @@
       </c>
       <c r="O65" s="3">
         <f>O63-O64</f>
-        <v>2403620</v>
+        <v>2436620</v>
       </c>
       <c r="P65" s="3">
         <f>P63-P64</f>
-        <v>230900</v>
+        <v>2335560</v>
       </c>
       <c r="Q65" s="3">
         <f>Q63-Q64</f>
-        <v>238500</v>
+        <v>2335560</v>
       </c>
     </row>
     <row r="66" spans="13:17" x14ac:dyDescent="0.45">
@@ -7892,15 +7870,15 @@
       </c>
       <c r="O66" s="3">
         <f>ROUNDDOWN(O65*0.021,0)</f>
-        <v>50476</v>
+        <v>51169</v>
       </c>
       <c r="P66" s="3">
         <f>ROUNDDOWN(P65*0.021,0)</f>
-        <v>4848</v>
+        <v>49046</v>
       </c>
       <c r="Q66" s="3">
         <f>ROUNDDOWN(Q65*0.021,0)</f>
-        <v>5008</v>
+        <v>49046</v>
       </c>
     </row>
     <row r="67" spans="13:17" x14ac:dyDescent="0.45">
@@ -7909,15 +7887,15 @@
       </c>
       <c r="O67" s="3">
         <f>ROUNDDOWN(SUM(O65:O66),0)</f>
-        <v>2454096</v>
+        <v>2487789</v>
       </c>
       <c r="P67" s="3">
         <f>ROUNDDOWN(SUM(P65:P66),0)</f>
-        <v>235748</v>
+        <v>2384606</v>
       </c>
       <c r="Q67" s="3">
         <f>ROUNDDOWN(SUM(Q65:Q66),0)</f>
-        <v>243508</v>
+        <v>2384606</v>
       </c>
     </row>
     <row r="68" spans="13:17" x14ac:dyDescent="0.45">
@@ -7943,15 +7921,15 @@
       </c>
       <c r="O69" s="3">
         <f>ROUNDDOWN(O67-O68,-2)</f>
-        <v>2454000</v>
+        <v>2487700</v>
       </c>
       <c r="P69" s="3">
         <f>ROUNDDOWN(P67-P68,-2)</f>
-        <v>235700</v>
+        <v>2384600</v>
       </c>
       <c r="Q69" s="3">
         <f>ROUNDDOWN(Q67-Q68,-2)</f>
-        <v>243500</v>
+        <v>2384600</v>
       </c>
     </row>
   </sheetData>
@@ -7980,7 +7958,8 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="2400" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -8006,30 +7985,30 @@
   <sheetData>
     <row r="2" spans="2:18" ht="19.8" x14ac:dyDescent="0.45">
       <c r="D2" s="20" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="M2" s="20" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.45">
       <c r="E4" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="G4" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="F4" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>253</v>
-      </c>
       <c r="N4" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="O4" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="P4" s="21" t="s">
         <v>251</v>
-      </c>
-      <c r="O4" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="P4" s="21" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="5" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -8037,7 +8016,7 @@
         <v>68</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D5" s="23"/>
       <c r="E5" s="24">
@@ -8045,11 +8024,11 @@
       </c>
       <c r="F5" s="25">
         <f>インプット表!K22</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
       <c r="G5" s="26">
         <f>+E5-F5</f>
-        <v>-48000</v>
+        <v>-464000</v>
       </c>
       <c r="H5" s="27"/>
       <c r="I5" s="27"/>
@@ -8057,7 +8036,7 @@
         <v>68</v>
       </c>
       <c r="L5" s="22" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="M5" s="23"/>
       <c r="N5" s="24">
@@ -8065,11 +8044,11 @@
       </c>
       <c r="O5" s="25">
         <f>インプット表!K22</f>
-        <v>48000</v>
+        <v>464000</v>
       </c>
       <c r="P5" s="59">
         <f>+N5-O5</f>
-        <v>-48000</v>
+        <v>-464000</v>
       </c>
       <c r="Q5" s="27"/>
       <c r="R5" s="27"/>
@@ -8077,15 +8056,15 @@
     <row r="6" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B6" s="71"/>
       <c r="C6" s="28" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E6" s="29">
         <f>計算結果!Q6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="F6" s="30">
         <f>+E6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="G6" s="31">
         <f>+E6-F6</f>
@@ -8095,15 +8074,15 @@
       <c r="I6" s="27"/>
       <c r="K6" s="71"/>
       <c r="L6" s="28" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="N6" s="29">
         <f>計算結果!Q6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="O6" s="30">
         <f>+N6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="P6" s="59">
         <f>+N6-O6</f>
@@ -8115,35 +8094,35 @@
     <row r="7" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B7" s="71"/>
       <c r="C7" s="22" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D7" s="23"/>
       <c r="E7" s="32">
         <f>計算結果!Q25</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="F7" s="33">
         <f>+E7+F5-2000</f>
-        <v>1716000</v>
+        <v>1779927</v>
       </c>
       <c r="G7" s="26">
         <f>+E7-F7</f>
-        <v>-46000</v>
+        <v>-462000</v>
       </c>
       <c r="H7" s="27"/>
       <c r="I7" s="27"/>
       <c r="K7" s="71"/>
       <c r="L7" s="22" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="M7" s="23"/>
       <c r="N7" s="32">
         <f>計算結果!Q25</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="O7" s="65">
         <f>計算結果!Q25</f>
-        <v>1670000</v>
+        <v>1317927</v>
       </c>
       <c r="P7" s="59">
         <f>+N7-O7</f>
@@ -8155,10 +8134,10 @@
     <row r="8" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B8" s="71"/>
       <c r="C8" s="83" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E8" s="35">
         <f>計算結果!Q29</f>
@@ -8176,10 +8155,10 @@
       <c r="I8" s="27"/>
       <c r="K8" s="71"/>
       <c r="L8" s="83" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="M8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="N8" s="35">
         <f>計算結果!Q29</f>
@@ -8200,7 +8179,7 @@
       <c r="B9" s="71"/>
       <c r="C9" s="83"/>
       <c r="D9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E9" s="34">
         <f>計算結果!Q31</f>
@@ -8219,7 +8198,7 @@
       <c r="K9" s="71"/>
       <c r="L9" s="83"/>
       <c r="M9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="N9" s="34">
         <f>計算結果!Q31</f>
@@ -8239,39 +8218,39 @@
     <row r="10" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B10" s="71"/>
       <c r="C10" s="80" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E10" s="37">
         <f>計算結果!Q50*1.021</f>
-        <v>243508.49999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="F10" s="37">
         <f>計算結果!P50*1.021</f>
-        <v>235748.89999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="G10" s="37">
         <f>E10-F10</f>
-        <v>7759.6000000000058</v>
+        <v>0</v>
       </c>
       <c r="H10" s="27"/>
       <c r="I10" s="27"/>
       <c r="K10" s="71"/>
       <c r="L10" s="80" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="N10" s="37">
         <f>計算結果!Q50*1.021</f>
-        <v>243508.49999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="O10" s="57">
         <f>計算結果!P50*1.021</f>
-        <v>235748.89999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="P10" s="60"/>
       <c r="Q10" s="27"/>
@@ -8281,7 +8260,7 @@
       <c r="B11" s="71"/>
       <c r="C11" s="81"/>
       <c r="D11" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E11" s="31">
         <f>E8*0.3*1.021</f>
@@ -8300,7 +8279,7 @@
       <c r="K11" s="71"/>
       <c r="L11" s="81"/>
       <c r="M11" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="N11" s="31">
         <f>N8*0.3*1.021</f>
@@ -8318,7 +8297,7 @@
       <c r="B12" s="71"/>
       <c r="C12" s="81"/>
       <c r="D12" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E12" s="31">
         <f>E9*0.15*1.021</f>
@@ -8337,7 +8316,7 @@
       <c r="K12" s="71"/>
       <c r="L12" s="81"/>
       <c r="M12" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="N12" s="31">
         <f>N9*0.15*1.021</f>
@@ -8355,43 +8334,43 @@
       <c r="B13" s="72"/>
       <c r="C13" s="82"/>
       <c r="D13" s="39" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E13" s="26">
         <f>SUM(E10:E12)</f>
-        <v>243508.49999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="F13" s="26">
         <f>SUM(F10:F12)</f>
-        <v>235748.89999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="G13" s="26">
         <f>E13-F13</f>
-        <v>7759.6000000000058</v>
+        <v>0</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I13" s="27"/>
       <c r="K13" s="72"/>
       <c r="L13" s="82"/>
       <c r="M13" s="39" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="N13" s="26">
         <f>SUM(N10:N12)</f>
-        <v>243508.49999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="O13" s="26">
         <f>SUM(O10:O12)</f>
-        <v>235748.89999999997</v>
+        <v>2384606.7599999998</v>
       </c>
       <c r="P13" s="26">
         <f>N13-O13</f>
-        <v>7759.6000000000058</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="40" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="R13" s="27"/>
     </row>
@@ -8412,16 +8391,16 @@
         <v>83</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="38">
         <f>計算結果!AB6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="F15" s="37">
         <f>+E15</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="G15" s="43">
         <f>+E15-F15</f>
@@ -8433,16 +8412,16 @@
         <v>83</v>
       </c>
       <c r="L15" s="41" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="M15" s="42"/>
       <c r="N15" s="38">
         <f>計算結果!AB6</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="O15" s="37">
         <f>+N15</f>
-        <v>5000000</v>
+        <v>13050000</v>
       </c>
       <c r="P15" s="59">
         <f>+N15-O15</f>
@@ -8454,23 +8433,23 @@
     <row r="16" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B16" s="71"/>
       <c r="C16" s="22" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D16" s="23"/>
       <c r="E16" s="33">
         <f>計算結果!AB24</f>
-        <v>1470000</v>
+        <v>1167927</v>
       </c>
       <c r="F16" s="26">
         <f>計算結果!AB24</f>
-        <v>1470000</v>
+        <v>1167927</v>
       </c>
       <c r="G16" s="24">
         <f>+E16-F16</f>
         <v>0</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I16" s="44">
         <f>計算結果!AB39</f>
@@ -8478,23 +8457,23 @@
       </c>
       <c r="K16" s="74"/>
       <c r="L16" s="22" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="M16" s="23"/>
       <c r="N16" s="33">
         <f>計算結果!AB24</f>
-        <v>1470000</v>
+        <v>1167927</v>
       </c>
       <c r="O16" s="26">
         <f>計算結果!AB24</f>
-        <v>1470000</v>
+        <v>1167927</v>
       </c>
       <c r="P16" s="59">
         <f>+N16-O16</f>
         <v>0</v>
       </c>
       <c r="Q16" s="27" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="R16" s="44">
         <f>計算結果!AB39</f>
@@ -8504,7 +8483,7 @@
     <row r="17" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B17" s="71"/>
       <c r="C17" s="76" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D17" s="45" t="s">
         <v>75</v>
@@ -8525,7 +8504,7 @@
       <c r="I17" s="27"/>
       <c r="K17" s="74"/>
       <c r="L17" s="76" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="M17" s="45" t="s">
         <v>75</v>
@@ -8588,18 +8567,18 @@
     <row r="19" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B19" s="71"/>
       <c r="C19" s="77" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D19" s="45" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E19" s="38">
         <f>(E15-E16)*0.1</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="F19" s="37">
         <f>(F15-F16)*0.1</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="G19" s="43">
         <f t="shared" ref="G19:G27" si="1">+E19-F19</f>
@@ -8609,18 +8588,18 @@
       <c r="I19" s="27"/>
       <c r="K19" s="74"/>
       <c r="L19" s="77" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="M19" s="45" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="N19" s="38">
         <f>(N15-N16)*0.1</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="O19" s="37">
         <f>(O15-O16)*0.1</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="P19" s="60">
         <f t="shared" ref="P19:P28" si="2">+N19-O19</f>
@@ -8633,7 +8612,7 @@
       <c r="B20" s="71"/>
       <c r="C20" s="78"/>
       <c r="D20" s="28" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E20" s="30">
         <f>E17*0.09</f>
@@ -8652,7 +8631,7 @@
       <c r="K20" s="74"/>
       <c r="L20" s="78"/>
       <c r="M20" s="28" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="N20" s="30">
         <f>N17*0.09</f>
@@ -8673,7 +8652,7 @@
       <c r="B21" s="71"/>
       <c r="C21" s="78"/>
       <c r="D21" s="28" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E21" s="30">
         <f>E18*0.05</f>
@@ -8692,7 +8671,7 @@
       <c r="K21" s="74"/>
       <c r="L21" s="78"/>
       <c r="M21" s="28" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="N21" s="30">
         <f>N18*0.05</f>
@@ -8717,11 +8696,11 @@
       </c>
       <c r="E22" s="33">
         <f>SUM(E19:E21)</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="F22" s="26">
         <f>SUM(F19:F21)</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="G22" s="24">
         <f t="shared" si="1"/>
@@ -8736,11 +8715,11 @@
       </c>
       <c r="N22" s="33">
         <f>SUM(N19:N21)</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="O22" s="26">
         <f>SUM(O19:O21)</f>
-        <v>353000</v>
+        <v>1188207.3</v>
       </c>
       <c r="P22" s="59">
         <f t="shared" si="2"/>
@@ -8752,7 +8731,7 @@
     <row r="23" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B23" s="71"/>
       <c r="C23" s="48" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D23" s="49"/>
       <c r="E23" s="30">
@@ -8771,7 +8750,7 @@
       <c r="I23" s="27"/>
       <c r="K23" s="74"/>
       <c r="L23" s="48" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="M23" s="49"/>
       <c r="N23" s="30">
@@ -8792,16 +8771,16 @@
     <row r="24" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B24" s="71"/>
       <c r="C24" s="50" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D24" s="51"/>
       <c r="E24" s="33">
         <f>E22-E23</f>
-        <v>350500</v>
+        <v>1185707.3</v>
       </c>
       <c r="F24" s="26">
         <f>F22-F23</f>
-        <v>350500</v>
+        <v>1185707.3</v>
       </c>
       <c r="G24" s="24">
         <f t="shared" si="1"/>
@@ -8811,16 +8790,16 @@
       <c r="I24" s="27"/>
       <c r="K24" s="74"/>
       <c r="L24" s="50" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="M24" s="51"/>
       <c r="N24" s="33">
         <f>N22-N23</f>
-        <v>350500</v>
+        <v>1185707.3</v>
       </c>
       <c r="O24" s="26">
         <f>O22-O23</f>
-        <v>350500</v>
+        <v>1185707.3</v>
       </c>
       <c r="P24" s="59">
         <f t="shared" si="2"/>
@@ -8832,115 +8811,115 @@
     <row r="25" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B25" s="71"/>
       <c r="C25" s="78" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E25" s="30">
         <v>0</v>
       </c>
       <c r="F25" s="31">
         <f>SUM(計算結果!W21:W22)</f>
-        <v>4600</v>
+        <v>46200</v>
       </c>
       <c r="G25" s="46">
         <f t="shared" si="1"/>
-        <v>-4600</v>
+        <v>-46200</v>
       </c>
       <c r="H25" s="27"/>
       <c r="I25" s="27"/>
       <c r="K25" s="74"/>
       <c r="L25" s="80" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="M25" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="N25">
         <v>0</v>
       </c>
       <c r="O25" s="56">
         <f>SUM(計算結果!W21:W22)</f>
-        <v>4600</v>
+        <v>46200</v>
       </c>
       <c r="P25" s="60">
         <f t="shared" si="2"/>
-        <v>-4600</v>
+        <v>-46200</v>
       </c>
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B26" s="71"/>
       <c r="C26" s="78"/>
       <c r="D26" s="28" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E26" s="30">
         <v>0</v>
       </c>
       <c r="F26" s="31">
         <f>SUM(計算結果!W30:W31)</f>
-        <v>36705</v>
+        <v>237140</v>
       </c>
       <c r="G26" s="46">
         <f t="shared" si="1"/>
-        <v>-36705</v>
+        <v>-237140</v>
       </c>
       <c r="H26" s="27"/>
       <c r="I26" s="27"/>
       <c r="K26" s="74"/>
       <c r="L26" s="81"/>
       <c r="M26" s="52" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="N26">
         <v>0</v>
       </c>
       <c r="O26" s="63">
         <f>SUM(計算結果!W30:W31)</f>
-        <v>36705</v>
+        <v>237140</v>
       </c>
       <c r="P26" s="62">
         <f t="shared" si="2"/>
-        <v>-36705</v>
+        <v>-237140</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B27" s="72"/>
       <c r="C27" s="79"/>
       <c r="D27" s="47" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E27" s="33">
         <v>0</v>
       </c>
       <c r="F27" s="26">
         <f>SUM(F25:F26)</f>
-        <v>41305</v>
+        <v>283340</v>
       </c>
       <c r="G27" s="24">
         <f t="shared" si="1"/>
-        <v>-41305</v>
+        <v>-283340</v>
       </c>
       <c r="H27" s="27" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I27" s="27"/>
       <c r="K27" s="74"/>
       <c r="L27" s="81"/>
       <c r="M27" s="53" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="N27">
         <v>0</v>
       </c>
       <c r="O27" s="63">
         <f>SUM(計算結果!W33:W34)</f>
-        <v>0</v>
+        <v>155662</v>
       </c>
       <c r="P27" s="61">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-155662</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.45">
@@ -8952,41 +8931,41 @@
       <c r="K28" s="75"/>
       <c r="L28" s="82"/>
       <c r="M28" s="47" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="N28" s="54">
         <v>0</v>
       </c>
       <c r="O28" s="59">
         <f>SUM(O25:O27)</f>
-        <v>41305</v>
+        <v>439002</v>
       </c>
       <c r="P28" s="59">
         <f t="shared" si="2"/>
-        <v>-41305</v>
+        <v>-439002</v>
       </c>
       <c r="Q28" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.45">
       <c r="D29" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E29" s="55">
         <f>E13+E22-E27</f>
-        <v>596508.5</v>
+        <v>3572814.0599999996</v>
       </c>
       <c r="F29" s="55">
         <f>F13+F22-F27</f>
-        <v>547443.89999999991</v>
+        <v>3289474.0599999996</v>
       </c>
       <c r="G29" s="26">
         <f>E29-F29</f>
-        <v>49064.600000000093</v>
+        <v>283340</v>
       </c>
       <c r="H29" s="27" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I29" s="27"/>
     </row>
@@ -8997,22 +8976,22 @@
       <c r="H30" s="27"/>
       <c r="I30" s="27"/>
       <c r="M30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="N30" s="55">
         <f>N13+N22-N28</f>
-        <v>596508.5</v>
+        <v>3572814.0599999996</v>
       </c>
       <c r="O30" s="55">
         <f>O13+O22-O28</f>
-        <v>547443.89999999991</v>
+        <v>3133812.0599999996</v>
       </c>
       <c r="P30" s="26">
         <f>N30-O30</f>
-        <v>49064.600000000093</v>
+        <v>439002</v>
       </c>
       <c r="Q30" s="27" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="R30" s="27"/>
     </row>
@@ -9130,7 +9109,7 @@
         <v>137</v>
       </c>
       <c r="X3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.45">
@@ -9217,10 +9196,10 @@
         <v>427500</v>
       </c>
       <c r="J5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="K5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L5" s="19">
         <v>7.1999999999999995E-2</v>
@@ -9286,7 +9265,7 @@
         <v>636000</v>
       </c>
       <c r="K6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="L6" s="1">
         <v>0.04</v>
@@ -9352,10 +9331,10 @@
         <v>1536000</v>
       </c>
       <c r="J7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="K7" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L7" s="1">
         <v>0.04</v>
@@ -9421,7 +9400,7 @@
         <v>2796000</v>
       </c>
       <c r="K8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="L8" s="19">
         <v>3.2000000000000001E-2</v>
@@ -9483,7 +9462,7 @@
         <v>4796000</v>
       </c>
       <c r="K9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L9" s="1">
         <v>0.04</v>
@@ -9520,7 +9499,7 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.45">
       <c r="K10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="L10" s="19">
         <v>3.2000000000000001E-2</v>
@@ -9554,7 +9533,7 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.45">
       <c r="K11" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L11" s="1">
         <v>0.04</v>
@@ -9585,7 +9564,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.45">
       <c r="J12" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="L12" s="1">
         <v>0.04</v>
@@ -9606,7 +9585,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.45">
       <c r="J13" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L13" s="1">
         <v>0.04</v>
@@ -9632,7 +9611,7 @@
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="J14" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="L14" s="1">
         <v>0.04</v>
@@ -9669,7 +9648,7 @@
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="J15" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L15" s="1">
         <v>0.04</v>
@@ -9705,7 +9684,7 @@
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="J16" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="L16" s="1">
         <v>0.08</v>
@@ -9736,7 +9715,7 @@
     </row>
     <row r="17" spans="10:22" x14ac:dyDescent="0.45">
       <c r="J17" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L17" s="1">
         <v>0.08</v>
@@ -9815,7 +9794,7 @@
     </row>
     <row r="20" spans="10:22" x14ac:dyDescent="0.45">
       <c r="J20" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L20">
         <v>0.8</v>
@@ -9832,7 +9811,7 @@
     </row>
     <row r="24" spans="10:22" x14ac:dyDescent="0.45">
       <c r="Q24" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="26" spans="10:22" x14ac:dyDescent="0.45">
@@ -9860,7 +9839,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -9871,23 +9850,23 @@
       </c>
       <c r="B2" s="3">
         <f>計算結果!W7</f>
-        <v>3530000</v>
+        <v>11882000</v>
       </c>
       <c r="C2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B3" s="3">
         <f>計算結果!W17+計算結果!W18</f>
-        <v>350500</v>
+        <v>1185700</v>
       </c>
       <c r="C3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B4" s="13" cm="1">
         <f t="array" ref="B4" xml:space="preserve">
@@ -9897,13 +9876,13 @@
   _xlpm.factor, マスター!$V$3:$V$9+0,
   _xlfn.XLOOKUP(_xlpm.x, _xlpm.lower, _xlpm.factor, , 1)
 )</f>
-        <v>0.69579999999999997</v>
+        <v>0.56306999999999996</v>
       </c>
       <c r="C4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B5" s="4">
         <v>0.9</v>
@@ -9917,14 +9896,14 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B8" s="3">
         <f xml:space="preserve">
@@ -9934,13 +9913,13 @@
   + 2000,
   0
 )</f>
-        <v>89855</v>
+        <v>423155</v>
       </c>
       <c r="C8"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B9" s="16">
         <f xml:space="preserve">
@@ -9950,7 +9929,7 @@
   + 2000,
   0
 )</f>
-        <v>89855</v>
+        <v>423155</v>
       </c>
       <c r="C9"/>
     </row>
@@ -9961,28 +9940,28 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B11"/>
       <c r="C11"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B12" s="3">
         <f>ROUND( VALUE(計算結果!$AB$6)*0.4 + 2000, 0 )</f>
-        <v>2002000</v>
+        <v>5222000</v>
       </c>
       <c r="C12"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B13" s="3">
         <f>ROUND( VALUE(計算結果!$AB$6)*0.3 + 2000, 0 )</f>
-        <v>1502000</v>
+        <v>3917000</v>
       </c>
       <c r="C13"/>
     </row>
@@ -9993,28 +9972,28 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B16" s="3">
         <f>MIN($B$8,$B$12,$B$13)</f>
-        <v>89855</v>
+        <v>423155</v>
       </c>
       <c r="C16"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B17" s="3">
         <f>MIN($B$9,$B$13)</f>
-        <v>89855</v>
+        <v>423155</v>
       </c>
       <c r="C17"/>
     </row>
@@ -10054,31 +10033,31 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C1" t="s">
         <v>68</v>
       </c>
       <c r="D1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" t="s">
+        <v>212</v>
+      </c>
+      <c r="O1" t="s">
+        <v>211</v>
+      </c>
+      <c r="P1" t="s">
         <v>210</v>
       </c>
-      <c r="E1" t="s">
-        <v>214</v>
-      </c>
-      <c r="O1" t="s">
-        <v>213</v>
-      </c>
-      <c r="P1" t="s">
-        <v>212</v>
-      </c>
       <c r="S1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="U1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.45">
@@ -10086,13 +10065,13 @@
         <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="P2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Q2">
         <v>0.05</v>
@@ -10108,13 +10087,13 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.45">
       <c r="D3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="P3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="Q3">
         <v>0.1</v>
@@ -10130,10 +10109,10 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.45">
       <c r="H4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="P4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="Q4">
         <v>0.2</v>
@@ -10149,10 +10128,10 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.45">
       <c r="G5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="P5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="Q5">
         <v>0.23</v>
@@ -10168,7 +10147,7 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="Q6">
         <v>0.33</v>
@@ -10184,7 +10163,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="Q7">
         <v>0.4</v>
@@ -10200,7 +10179,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="Q8">
         <v>0.45</v>
@@ -10220,7 +10199,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.45">
       <c r="O10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="P10" t="s">
         <v>138</v>
@@ -10247,31 +10226,31 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.45">
       <c r="O13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="P13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="S13" s="18"/>
       <c r="U13" s="18"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="S14" s="18"/>
       <c r="U14" s="18"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P15" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="S15" s="18"/>
       <c r="U15" s="18"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.45">
       <c r="P16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="S16" s="18"/>
       <c r="U16" s="18"/>
@@ -10282,10 +10261,10 @@
     </row>
     <row r="18" spans="15:21" x14ac:dyDescent="0.45">
       <c r="O18" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="P18" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="S18" s="18"/>
       <c r="U18" s="18"/>
@@ -10388,7 +10367,7 @@
     </row>
     <row r="25" spans="15:21" x14ac:dyDescent="0.45">
       <c r="P25" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
wip: ensure local tree is clean for v0.5 sync
</commit_message>
<xml_diff>
--- a/tests/Fixtures/個人住民税vol23.xlsx
+++ b/tests/Fixtures/個人住民税vol23.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4245ae31b7bca767/Desktop/ふるさと納税クラウド/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{E8F1E613-22D3-4668-A0D3-EEF16E5E6BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A72DF1B8-8E30-497E-A581-282B3B8A1B07}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{E8F1E613-22D3-4668-A0D3-EEF16E5E6BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5FAC136-59CB-4485-8E20-EFBF6314E32E}"/>
   <bookViews>
-    <workbookView xWindow="12672" yWindow="756" windowWidth="16128" windowHeight="15432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="336" yWindow="528" windowWidth="16128" windowHeight="15432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="インプット表" sheetId="1" r:id="rId1"/>
@@ -250,7 +250,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="286">
   <si>
     <t>前期</t>
   </si>
@@ -2436,9 +2436,6 @@
       <t>ガク</t>
     </rPh>
     <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>INDEX(マスター!$D$3:$D$9,MATCH(1,(P41&gt;=マスター!$A$3:$A$9)*(P41&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</t>
   </si>
   <si>
     <t>特定親族特別控除</t>
@@ -2980,6 +2977,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="255"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="255"/>
     </xf>
@@ -3000,18 +3009,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3494,7 +3491,7 @@
     <col min="8" max="8" width="24.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.19921875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.3984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.45">
@@ -3531,7 +3528,7 @@
         <v>703890</v>
       </c>
       <c r="K2" s="12">
-        <v>327927</v>
+        <v>50000000</v>
       </c>
       <c r="P2" s="6"/>
       <c r="Q2" t="s">
@@ -3724,13 +3721,13 @@
         <v>18</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K18" s="3">
         <v>1000000</v>
       </c>
       <c r="M18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
@@ -4048,19 +4045,19 @@
       </c>
       <c r="W7" s="3">
         <f>IF(ROUNDDOWN(AB6-AB24,-3)&lt;0,0,ROUNDDOWN(AB6-AB24,-3))</f>
-        <v>11882000</v>
+        <v>0</v>
       </c>
       <c r="X7" s="3">
         <f>IF(ROUNDDOWN(AB6-AB24,-3)&lt;0,0,ROUNDDOWN(AB6-AB24,-3))</f>
-        <v>11882000</v>
+        <v>0</v>
       </c>
       <c r="Z7"/>
       <c r="AD7" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="AE7" s="3">
+      <c r="AE7" s="3" t="e">
         <f>W38</f>
-        <v>439002</v>
+        <v>#N/A</v>
       </c>
       <c r="AF7" s="3"/>
     </row>
@@ -4123,11 +4120,11 @@
       </c>
       <c r="P8" s="3">
         <f>インプット表!K2</f>
-        <v>327927</v>
+        <v>50000000</v>
       </c>
       <c r="Q8" s="3">
         <f>インプット表!K2</f>
-        <v>327927</v>
+        <v>50000000</v>
       </c>
       <c r="T8" t="s">
         <v>177</v>
@@ -4152,14 +4149,14 @@
       </c>
       <c r="AB8" s="3">
         <f t="shared" si="0"/>
-        <v>327927</v>
+        <v>50000000</v>
       </c>
       <c r="AD8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="AE8" s="3">
+      <c r="AE8" s="3" t="e">
         <f>SUM(AE6:AE7)</f>
-        <v>439002</v>
+        <v>#N/A</v>
       </c>
       <c r="AF8" s="3"/>
       <c r="AG8" s="5"/>
@@ -4376,7 +4373,7 @@
   +P37*IF(W6=TRUE,マスター!$L$15,マスター!$N$15)
   +P38*IF(W6=TRUE,マスター!$L$16,マスター!$N$16)
   +P39*IF(W6=TRUE,マスター!$L$17,マスター!$N$17)</f>
-        <v>712920</v>
+        <v>0</v>
       </c>
       <c r="X11" s="3">
         <f>X7*IF(X6=TRUE,マスター!$L$4,マスター!$N$4)
@@ -4393,7 +4390,7 @@
   +Q37*IF(X6=TRUE,マスター!$L$15,マスター!$N$15)
   +Q38*IF(X6=TRUE,マスター!$L$16,マスター!$N$16)
   +Q39*IF(X6=TRUE,マスター!$L$17,マスター!$N$17)</f>
-        <v>712920</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="s">
         <v>12</v>
@@ -4473,7 +4470,7 @@
   +P37*IF(W6=TRUE,マスター!$M$15,マスター!$O$15)
   +P38*IF(W6=TRUE,マスター!$M$16,マスター!$O$16)
   +P39*IF(W6=TRUE,マスター!$M$17,マスター!$O$17)</f>
-        <v>475280</v>
+        <v>0</v>
       </c>
       <c r="X12" s="3">
         <f>X7*IF(X6=TRUE,マスター!$M$4,マスター!$O$4)
@@ -4490,7 +4487,7 @@
   +Q37*IF(X6=TRUE,マスター!$M$15,マスター!$O$15)
   +Q38*IF(X6=TRUE,マスター!$M$16,マスター!$O$16)
   +Q39*IF(X6=TRUE,マスター!$M$17,マスター!$O$17)</f>
-        <v>475280</v>
+        <v>0</v>
       </c>
       <c r="Z12" t="s">
         <v>14</v>
@@ -4703,11 +4700,11 @@
       </c>
       <c r="W14" s="3">
         <f>IF(W7=0,0,50000*IF(W6=TRUE,マスター!$L$18,マスター!$N$18))</f>
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="X14" s="3">
         <f>IF(X7=0,0,50000*IF(X6=TRUE,マスター!$L$18,マスター!$N$18))</f>
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="s">
         <v>19</v>
@@ -4815,11 +4812,11 @@
       </c>
       <c r="W15" s="3">
         <f>IF(W7=0,0,50000*IF(W6=TRUE,マスター!$M$18,マスター!$O$18))</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="X15" s="3">
         <f>IF(X7=0,0,50000*IF(X6=TRUE,マスター!$M$18,マスター!$O$18))</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="s">
         <v>47</v>
@@ -5098,11 +5095,11 @@
       </c>
       <c r="W17" s="3">
         <f t="shared" ref="W17:X18" si="3">W11-W14</f>
-        <v>711420</v>
+        <v>0</v>
       </c>
       <c r="X17" s="3">
         <f t="shared" si="3"/>
-        <v>711420</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="s">
         <v>229</v>
@@ -5210,11 +5207,11 @@
       </c>
       <c r="W18" s="3">
         <f>W12-W15</f>
-        <v>474280</v>
+        <v>0</v>
       </c>
       <c r="X18" s="3">
         <f t="shared" si="3"/>
-        <v>474280</v>
+        <v>0</v>
       </c>
       <c r="Z18" t="s">
         <v>33</v>
@@ -5237,7 +5234,7 @@
         <v>13831070</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O19" s="3" cm="1">
         <f t="array" ref="O19">IF(O6=0,0,INDEX({0,630000,610000,510000,410000,310000,210000,110000,60000,30000,0},
@@ -5263,14 +5260,14 @@
       </c>
       <c r="W19" s="3">
         <f>SUM(W17:W18)</f>
-        <v>1185700</v>
+        <v>0</v>
       </c>
       <c r="X19" s="3">
         <f>SUM(X17:X18)</f>
-        <v>1185700</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AA19" s="3">
         <v>0</v>
@@ -5373,31 +5370,31 @@
       </c>
       <c r="P21" s="3">
         <f>SUM(P8:P20)</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="Q21" s="3">
         <f>SUM(Q8:Q20)</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="U21" t="s">
         <v>45</v>
       </c>
       <c r="V21" s="3">
-        <f>IF(N(インプット表!$J$30)&lt;=2000,0,
+        <f>MAX(IF(N(インプット表!$J$30)&lt;=2000,0,
       (MIN(N(インプット表!$J$30), N(AA6)*0.3)-2000)
-      *IF($V$6=TRUE, マスター!$L$19, マスター!$N$19))</f>
+      *IF($V$6=TRUE, マスター!$L$19, マスター!$N$19)),0)</f>
         <v>26760</v>
       </c>
       <c r="W21" s="3">
-        <f>IF(N(インプット表!$K$30)&lt;=2000,0,
+        <f>MAX(IF(N(インプット表!$K$30)&lt;=2000,0,
       (MIN(N(インプット表!$K$30), SUM(Q42:Q48)*0.3)-2000)
-      *IF($W$6=TRUE, マスター!$L$19, マスター!$N$19))</f>
-        <v>27720</v>
+      *IF($W$6=TRUE, マスター!$L$19, マスター!$N$19)),0)</f>
+        <v>0</v>
       </c>
       <c r="X21" s="12">
-        <f xml:space="preserve"> IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
+        <f>MAX( IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
           ( MIN( N(インプット表!$K$30 - インプット表!$K$22), N(AB6)*0.3 ) - 2000 )
-          * IF($W$6, マスター!$L$19, マスター!$N$19) )</f>
+          * IF($W$6, マスター!$L$19, マスター!$N$19) ),0)</f>
         <v>0</v>
       </c>
       <c r="Z21" t="s">
@@ -5477,21 +5474,21 @@
         <v>46</v>
       </c>
       <c r="V22" s="3">
-        <f>IF(N(インプット表!$J$30)&lt;=2000,0,
+        <f>MAX(IF(N(インプット表!$J$30)&lt;=2000,0,
        (MIN(N(インプット表!$J$30), N(AA6)*0.3)-2000)
-       *IF($V$6=TRUE, マスター!$M$19, マスター!$O$19))</f>
+       *IF($V$6=TRUE, マスター!$M$19, マスター!$O$19)),0)</f>
         <v>17840</v>
       </c>
       <c r="W22" s="3">
-        <f>IF(N(インプット表!$K$30)&lt;=2000,0,
+        <f>MAX(IF(N(インプット表!$K$30)&lt;=2000,0,
        (MIN(N(インプット表!$K$30), SUM(Q42:Q48)*0.3)-2000)
-       *IF($W$6=TRUE, マスター!$M$19, マスター!$O$19))</f>
-        <v>18480</v>
+       *IF($W$6=TRUE, マスター!$M$19, マスター!$O$19)),0)</f>
+        <v>0</v>
       </c>
       <c r="X22" s="12">
-        <f xml:space="preserve"> IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
+        <f>MAX( IF( N(インプット表!$K$30 - インプット表!$K$22) &lt;= 2000, 0,
           ( MIN( N(インプット表!$K$30 - インプット表!$K$22), N(AB6)*0.3 ) - 2000 )
-          * IF($W$6, マスター!$M$19, マスター!$O$19) )</f>
+          * IF($W$6, マスター!$M$19, マスター!$O$19) ),0)</f>
         <v>0</v>
       </c>
       <c r="Z22" s="3" t="s">
@@ -5661,12 +5658,12 @@
 )</f>
         <v>150677.53199999998</v>
       </c>
-      <c r="W24" s="3">
+      <c r="W24" s="3" t="e">
         <f xml:space="preserve">
 IF(N(インプット表!$K$31)&lt;=2000, 0,
    (N(インプット表!$K$31)-2000) * $AB$56 * IF($W$6, マスター!$L$20, マスター!$N$20)
 )</f>
-        <v>156083.00399999999</v>
+        <v>#N/A</v>
       </c>
       <c r="X24" s="12">
         <v>0</v>
@@ -5680,7 +5677,7 @@
       </c>
       <c r="AB24" s="3">
         <f>SUM(AB8:AB23)</f>
-        <v>1167927</v>
+        <v>50840000</v>
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.45">
@@ -5748,11 +5745,11 @@
       </c>
       <c r="P25" s="3">
         <f>SUM(P21:P24)</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="Q25" s="3">
         <f>SUM(Q21:Q24)</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="U25" t="s">
         <v>46</v>
@@ -5764,12 +5761,12 @@
 )</f>
         <v>100451.68799999999</v>
       </c>
-      <c r="W25" s="3">
+      <c r="W25" s="3" t="e">
         <f xml:space="preserve">
 IF(N(インプット表!$K$31)&lt;=2000, 0,
    (N(インプット表!$K$31)-2000) * $AB$56 * IF($W$6, マスター!$M$20, マスター!$O$20)
 )</f>
-        <v>104055.336</v>
+        <v>#N/A</v>
       </c>
       <c r="X25" s="12">
         <v>0</v>
@@ -5815,7 +5812,7 @@
       </c>
       <c r="W27" s="3">
         <f>N($W$17)*0.2</f>
-        <v>142284</v>
+        <v>0</v>
       </c>
       <c r="X27" s="12">
         <v>0</v>
@@ -5856,7 +5853,7 @@
       </c>
       <c r="W28" s="3">
         <f>N($W$18)*0.2</f>
-        <v>94856</v>
+        <v>0</v>
       </c>
       <c r="X28" s="12">
         <v>0</v>
@@ -5914,9 +5911,9 @@
         <f>MIN(N($V$24), N($V$27))</f>
         <v>150456</v>
       </c>
-      <c r="W30" s="3">
+      <c r="W30" s="3" t="e">
         <f>ROUNDUP(MIN(N($W$24), N($W$27)),0)</f>
-        <v>142284</v>
+        <v>#N/A</v>
       </c>
       <c r="X30" s="12">
         <v>0</v>
@@ -5960,9 +5957,9 @@
         <f>MIN(N($V$25), N($V$28))</f>
         <v>100304</v>
       </c>
-      <c r="W31" s="3">
+      <c r="W31" s="3" t="e">
         <f>ROUNDUP(MIN(N($W$25),N($W$28)),0)</f>
-        <v>94856</v>
+        <v>#N/A</v>
       </c>
       <c r="X31" s="12">
         <v>0</v>
@@ -6055,14 +6052,14 @@
 ),0)</f>
         <v>0</v>
       </c>
-      <c r="W33" s="5" cm="1">
+      <c r="W33" s="5" t="e" cm="1">
         <f t="array" ref="W33" xml:space="preserve">
 ROUNDUP(
 IF($W$32,
 MAX(0,N(インプット表!$K$31)-2000)*AB56*INDEX(マスター!$AA$4:$AA$8,MATCH(1,(計算結果!$AB$49&gt;=マスター!$X$4:$X$8)*(計算結果!$AB$49&lt;=IF(マスター!$Z$4:$Z$8="",1E+99,マスター!$Z$4:$Z$8)),0))*IF($W$6,4/5,3/5),
 0
 ),0)</f>
-        <v>93397</v>
+        <v>#N/A</v>
       </c>
       <c r="X33" s="12">
         <v>0</v>
@@ -6124,7 +6121,7 @@
 ),0)</f>
         <v>0</v>
       </c>
-      <c r="W34" s="5" cm="1">
+      <c r="W34" s="5" t="e" cm="1">
         <f t="array" ref="W34" xml:space="preserve">
 ROUNDUP(
 IF($W$32,
@@ -6132,7 +6129,7 @@
 N($W$18)*0.2),
 0
 ),0)</f>
-        <v>62265</v>
+        <v>#N/A</v>
       </c>
       <c r="X34" s="12">
         <v>0</v>
@@ -6295,9 +6292,9 @@
         <f>ROUNDUP($V$21+IF($V$32,$V$33,$V$30),0)</f>
         <v>177216</v>
       </c>
-      <c r="W36" s="3">
+      <c r="W36" s="3" t="e">
         <f>ROUNDUP($W$21+$W$33+$W$30,0)</f>
-        <v>263401</v>
+        <v>#N/A</v>
       </c>
       <c r="X36" s="12">
         <f>ROUNDDOWN(X21+X33,-2)</f>
@@ -6380,9 +6377,9 @@
         <f>ROUNDUP($V$22+IF($V$32,$V$34,$V$31),0)</f>
         <v>118144</v>
       </c>
-      <c r="W37" s="3">
+      <c r="W37" s="3" t="e">
         <f>ROUNDUP($W$22+$W$34+$W$31,0)</f>
-        <v>175601</v>
+        <v>#N/A</v>
       </c>
       <c r="X37" s="12">
         <f>ROUNDDOWN(X22+X34,-2)</f>
@@ -6423,9 +6420,9 @@
         <f>SUM(V36:V37)</f>
         <v>295360</v>
       </c>
-      <c r="W38" s="3">
+      <c r="W38" s="3" t="e">
         <f>SUM(W36:W37)</f>
-        <v>439002</v>
+        <v>#N/A</v>
       </c>
       <c r="X38" s="12">
         <f>SUM(X36:X37)</f>
@@ -6650,11 +6647,11 @@
       </c>
       <c r="P41" s="3">
         <f>MIN(P25, P40)</f>
-        <v>1317927</v>
+        <v>13050000</v>
       </c>
       <c r="Q41" s="3">
-        <f>Q25</f>
-        <v>1317927</v>
+        <f>MIN(Q25, Q40)</f>
+        <v>13050000</v>
       </c>
       <c r="T41"/>
       <c r="Z41" t="s">
@@ -6736,11 +6733,11 @@
       </c>
       <c r="P42" s="3">
         <f>ROUNDDOWN(P40 - P41,-3)</f>
-        <v>11732000</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="3">
         <f>ROUNDDOWN(Q40 - Q41,-3)</f>
-        <v>11732000</v>
+        <v>0</v>
       </c>
       <c r="T42"/>
       <c r="Z42" t="s">
@@ -6752,7 +6749,7 @@
       </c>
       <c r="AB42" s="5">
         <f>INDEX($P:$P, MATCH("総合課税",$M:$M,0))</f>
-        <v>11732000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.45">
@@ -7192,7 +7189,7 @@
       </c>
       <c r="AB49" s="14">
         <f>AB42-$AB$39</f>
-        <v>11682000</v>
+        <v>-50000</v>
       </c>
     </row>
     <row r="50" spans="1:32" x14ac:dyDescent="0.45">
@@ -7267,11 +7264,11 @@
       </c>
       <c r="P50" s="3" cm="1">
         <f t="array" ref="P50">P42*INDEX(マスター!$D$3:$D$9,MATCH(1,(P42&gt;=マスター!$A$3:$A$9)*(P42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))-INDEX(マスター!$E$3:$E$9,MATCH(1,(P42&gt;=マスター!$A$3:$A$9)*(P42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
       <c r="Q50" s="3" cm="1">
         <f t="array" ref="Q50">Q42*INDEX(マスター!$D$3:$D$9,MATCH(1,(Q42&gt;=マスター!$A$3:$A$9)*(Q42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))-INDEX(マスター!$E$3:$E$9,MATCH(1,(Q42&gt;=マスター!$A$3:$A$9)*(Q42&lt;=IF(マスター!$C$3:$C$9="",1E+99,マスター!$C$3:$C$9)),0))</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
       <c r="Z50" t="s">
         <v>156</v>
@@ -7280,9 +7277,9 @@
         <f xml:space="preserve"> _xlfn.XLOOKUP(MAX(0, $AA$49), マスター!$S$4:$S$10, マスター!$V$4:$V$10, , 1)</f>
         <v>0.56306999999999996</v>
       </c>
-      <c r="AB50">
+      <c r="AB50" t="e">
         <f>LOOKUP($AB$49, マスター!$Q$4:$Q$10, マスター!$V$4:$V$10)</f>
-        <v>0.56306999999999996</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="51" spans="1:32" x14ac:dyDescent="0.45">
@@ -7607,14 +7604,14 @@
 )</f>
         <v>0.56306999999999996</v>
       </c>
-      <c r="AB56" s="15">
+      <c r="AB56" s="15" t="e">
         <f xml:space="preserve">
 MIN(  $AB$50,
   IF(AND($AB$49&lt;0, N($AB$43)=0, N($AB$44)=0), $AB$51, 1),
   IF($AB$54&lt;&gt;"", $AB$54, 1),
   IF($AB$55&lt;&gt;"", $AB$55, 1)
 )</f>
-        <v>0.56306999999999996</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="57" spans="1:32" x14ac:dyDescent="0.45">
@@ -7644,11 +7641,11 @@
       </c>
       <c r="P59" s="3">
         <f>ROUNDDOWN(SUM(P50:P57),0)</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
       <c r="Q59" s="3">
         <f>ROUNDDOWN(SUM(Q50:Q57),0)</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:32" x14ac:dyDescent="0.45">
@@ -7823,11 +7820,11 @@
       </c>
       <c r="P63" s="3">
         <f>P59-SUM(P60:P62)</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
       <c r="Q63" s="3">
         <f>Q59-SUM(Q60:Q62)</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:32" x14ac:dyDescent="0.45">
@@ -7857,11 +7854,11 @@
       </c>
       <c r="P65" s="3">
         <f>P63-P64</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
       <c r="Q65" s="3">
         <f>Q63-Q64</f>
-        <v>2335560</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="13:17" x14ac:dyDescent="0.45">
@@ -7874,11 +7871,11 @@
       </c>
       <c r="P66" s="3">
         <f>ROUNDDOWN(P65*0.021,0)</f>
-        <v>49046</v>
+        <v>0</v>
       </c>
       <c r="Q66" s="3">
         <f>ROUNDDOWN(Q65*0.021,0)</f>
-        <v>49046</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="13:17" x14ac:dyDescent="0.45">
@@ -7891,11 +7888,11 @@
       </c>
       <c r="P67" s="3">
         <f>ROUNDDOWN(SUM(P65:P66),0)</f>
-        <v>2384606</v>
+        <v>0</v>
       </c>
       <c r="Q67" s="3">
         <f>ROUNDDOWN(SUM(Q65:Q66),0)</f>
-        <v>2384606</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="13:17" x14ac:dyDescent="0.45">
@@ -7925,11 +7922,11 @@
       </c>
       <c r="P69" s="3">
         <f>ROUNDDOWN(P67-P68,-2)</f>
-        <v>2384600</v>
+        <v>0</v>
       </c>
       <c r="Q69" s="3">
         <f>ROUNDDOWN(Q67-Q68,-2)</f>
-        <v>2384600</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8099,11 +8096,11 @@
       <c r="D7" s="23"/>
       <c r="E7" s="32">
         <f>計算結果!Q25</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="F7" s="33">
         <f>+E7+F5-2000</f>
-        <v>1779927</v>
+        <v>51452000</v>
       </c>
       <c r="G7" s="26">
         <f>+E7-F7</f>
@@ -8118,11 +8115,11 @@
       <c r="M7" s="23"/>
       <c r="N7" s="32">
         <f>計算結果!Q25</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="O7" s="65">
         <f>計算結果!Q25</f>
-        <v>1317927</v>
+        <v>50990000</v>
       </c>
       <c r="P7" s="59">
         <f>+N7-O7</f>
@@ -8133,7 +8130,7 @@
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B8" s="71"/>
-      <c r="C8" s="83" t="s">
+      <c r="C8" s="73" t="s">
         <v>255</v>
       </c>
       <c r="D8" t="s">
@@ -8154,7 +8151,7 @@
       <c r="H8" s="27"/>
       <c r="I8" s="27"/>
       <c r="K8" s="71"/>
-      <c r="L8" s="83" t="s">
+      <c r="L8" s="73" t="s">
         <v>255</v>
       </c>
       <c r="M8" t="s">
@@ -8177,7 +8174,7 @@
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B9" s="71"/>
-      <c r="C9" s="83"/>
+      <c r="C9" s="73"/>
       <c r="D9" t="s">
         <v>257</v>
       </c>
@@ -8196,7 +8193,7 @@
       <c r="H9" s="27"/>
       <c r="I9" s="27"/>
       <c r="K9" s="71"/>
-      <c r="L9" s="83"/>
+      <c r="L9" s="73"/>
       <c r="M9" t="s">
         <v>257</v>
       </c>
@@ -8217,7 +8214,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B10" s="71"/>
-      <c r="C10" s="80" t="s">
+      <c r="C10" s="74" t="s">
         <v>258</v>
       </c>
       <c r="D10" s="36" t="s">
@@ -8225,11 +8222,11 @@
       </c>
       <c r="E10" s="37">
         <f>計算結果!Q50*1.021</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="F10" s="37">
         <f>計算結果!P50*1.021</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="G10" s="37">
         <f>E10-F10</f>
@@ -8238,7 +8235,7 @@
       <c r="H10" s="27"/>
       <c r="I10" s="27"/>
       <c r="K10" s="71"/>
-      <c r="L10" s="80" t="s">
+      <c r="L10" s="74" t="s">
         <v>258</v>
       </c>
       <c r="M10" s="36" t="s">
@@ -8246,11 +8243,11 @@
       </c>
       <c r="N10" s="37">
         <f>計算結果!Q50*1.021</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="O10" s="57">
         <f>計算結果!P50*1.021</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="P10" s="60"/>
       <c r="Q10" s="27"/>
@@ -8258,7 +8255,7 @@
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B11" s="71"/>
-      <c r="C11" s="81"/>
+      <c r="C11" s="75"/>
       <c r="D11" t="s">
         <v>260</v>
       </c>
@@ -8277,7 +8274,7 @@
       <c r="H11" s="27"/>
       <c r="I11" s="27"/>
       <c r="K11" s="71"/>
-      <c r="L11" s="81"/>
+      <c r="L11" s="75"/>
       <c r="M11" t="s">
         <v>260</v>
       </c>
@@ -8295,7 +8292,7 @@
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B12" s="71"/>
-      <c r="C12" s="81"/>
+      <c r="C12" s="75"/>
       <c r="D12" t="s">
         <v>261</v>
       </c>
@@ -8314,7 +8311,7 @@
       <c r="H12" s="27"/>
       <c r="I12" s="27"/>
       <c r="K12" s="71"/>
-      <c r="L12" s="81"/>
+      <c r="L12" s="75"/>
       <c r="M12" t="s">
         <v>261</v>
       </c>
@@ -8332,17 +8329,17 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B13" s="72"/>
-      <c r="C13" s="82"/>
+      <c r="C13" s="76"/>
       <c r="D13" s="39" t="s">
         <v>262</v>
       </c>
       <c r="E13" s="26">
         <f>SUM(E10:E12)</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="F13" s="26">
         <f>SUM(F10:F12)</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="G13" s="26">
         <f>E13-F13</f>
@@ -8353,17 +8350,17 @@
       </c>
       <c r="I13" s="27"/>
       <c r="K13" s="72"/>
-      <c r="L13" s="82"/>
+      <c r="L13" s="76"/>
       <c r="M13" s="39" t="s">
         <v>262</v>
       </c>
       <c r="N13" s="26">
         <f>SUM(N10:N12)</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="O13" s="26">
         <f>SUM(O10:O12)</f>
-        <v>2384606.7599999998</v>
+        <v>0</v>
       </c>
       <c r="P13" s="26">
         <f>N13-O13</f>
@@ -8408,7 +8405,7 @@
       </c>
       <c r="H15" s="27"/>
       <c r="I15" s="27"/>
-      <c r="K15" s="73" t="s">
+      <c r="K15" s="77" t="s">
         <v>83</v>
       </c>
       <c r="L15" s="41" t="s">
@@ -8438,11 +8435,11 @@
       <c r="D16" s="23"/>
       <c r="E16" s="33">
         <f>計算結果!AB24</f>
-        <v>1167927</v>
+        <v>50840000</v>
       </c>
       <c r="F16" s="26">
         <f>計算結果!AB24</f>
-        <v>1167927</v>
+        <v>50840000</v>
       </c>
       <c r="G16" s="24">
         <f>+E16-F16</f>
@@ -8455,18 +8452,18 @@
         <f>計算結果!AB39</f>
         <v>50000</v>
       </c>
-      <c r="K16" s="74"/>
+      <c r="K16" s="78"/>
       <c r="L16" s="22" t="s">
         <v>266</v>
       </c>
       <c r="M16" s="23"/>
       <c r="N16" s="33">
         <f>計算結果!AB24</f>
-        <v>1167927</v>
+        <v>50840000</v>
       </c>
       <c r="O16" s="26">
         <f>計算結果!AB24</f>
-        <v>1167927</v>
+        <v>50840000</v>
       </c>
       <c r="P16" s="59">
         <f>+N16-O16</f>
@@ -8482,7 +8479,7 @@
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B17" s="71"/>
-      <c r="C17" s="76" t="s">
+      <c r="C17" s="80" t="s">
         <v>268</v>
       </c>
       <c r="D17" s="45" t="s">
@@ -8502,8 +8499,8 @@
       </c>
       <c r="H17" s="27"/>
       <c r="I17" s="27"/>
-      <c r="K17" s="74"/>
-      <c r="L17" s="76" t="s">
+      <c r="K17" s="78"/>
+      <c r="L17" s="80" t="s">
         <v>268</v>
       </c>
       <c r="M17" s="45" t="s">
@@ -8526,7 +8523,7 @@
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B18" s="71"/>
-      <c r="C18" s="76"/>
+      <c r="C18" s="80"/>
       <c r="D18" s="28" t="s">
         <v>76</v>
       </c>
@@ -8544,8 +8541,8 @@
       </c>
       <c r="H18" s="27"/>
       <c r="I18" s="27"/>
-      <c r="K18" s="74"/>
-      <c r="L18" s="76"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="80"/>
       <c r="M18" s="28" t="s">
         <v>76</v>
       </c>
@@ -8566,51 +8563,51 @@
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B19" s="71"/>
-      <c r="C19" s="77" t="s">
+      <c r="C19" s="81" t="s">
         <v>269</v>
       </c>
       <c r="D19" s="45" t="s">
         <v>270</v>
       </c>
       <c r="E19" s="38">
-        <f>(E15-E16)*0.1</f>
-        <v>1188207.3</v>
+        <f>計算結果!AA42*0.1</f>
+        <v>1205400</v>
       </c>
       <c r="F19" s="37">
-        <f>(F15-F16)*0.1</f>
-        <v>1188207.3</v>
+        <f>計算結果!AB42*0.1</f>
+        <v>0</v>
       </c>
       <c r="G19" s="43">
         <f t="shared" ref="G19:G27" si="1">+E19-F19</f>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="H19" s="27"/>
       <c r="I19" s="27"/>
-      <c r="K19" s="74"/>
-      <c r="L19" s="77" t="s">
+      <c r="K19" s="78"/>
+      <c r="L19" s="81" t="s">
         <v>269</v>
       </c>
       <c r="M19" s="45" t="s">
         <v>270</v>
       </c>
       <c r="N19" s="38">
-        <f>(N15-N16)*0.1</f>
-        <v>1188207.3</v>
+        <f>計算結果!AA42*0.1</f>
+        <v>1205400</v>
       </c>
       <c r="O19" s="37">
-        <f>(O15-O16)*0.1</f>
-        <v>1188207.3</v>
+        <f>計算結果!AB42*0.1</f>
+        <v>0</v>
       </c>
       <c r="P19" s="60">
         <f t="shared" ref="P19:P28" si="2">+N19-O19</f>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="Q19" s="27"/>
       <c r="R19" s="27"/>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B20" s="71"/>
-      <c r="C20" s="78"/>
+      <c r="C20" s="82"/>
       <c r="D20" s="28" t="s">
         <v>271</v>
       </c>
@@ -8628,8 +8625,8 @@
       </c>
       <c r="H20" s="27"/>
       <c r="I20" s="27"/>
-      <c r="K20" s="74"/>
-      <c r="L20" s="78"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="82"/>
       <c r="M20" s="28" t="s">
         <v>271</v>
       </c>
@@ -8650,7 +8647,7 @@
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B21" s="71"/>
-      <c r="C21" s="78"/>
+      <c r="C21" s="82"/>
       <c r="D21" s="28" t="s">
         <v>272</v>
       </c>
@@ -8668,8 +8665,8 @@
       </c>
       <c r="H21" s="27"/>
       <c r="I21" s="27"/>
-      <c r="K21" s="74"/>
-      <c r="L21" s="78"/>
+      <c r="K21" s="78"/>
+      <c r="L21" s="82"/>
       <c r="M21" s="28" t="s">
         <v>272</v>
       </c>
@@ -8690,40 +8687,40 @@
     </row>
     <row r="22" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B22" s="71"/>
-      <c r="C22" s="79"/>
+      <c r="C22" s="83"/>
       <c r="D22" s="47" t="s">
         <v>48</v>
       </c>
       <c r="E22" s="33">
         <f>SUM(E19:E21)</f>
-        <v>1188207.3</v>
+        <v>1205400</v>
       </c>
       <c r="F22" s="26">
         <f>SUM(F19:F21)</f>
-        <v>1188207.3</v>
+        <v>0</v>
       </c>
       <c r="G22" s="24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="H22" s="27"/>
       <c r="I22" s="27"/>
-      <c r="K22" s="74"/>
-      <c r="L22" s="79"/>
+      <c r="K22" s="78"/>
+      <c r="L22" s="83"/>
       <c r="M22" s="47" t="s">
         <v>48</v>
       </c>
       <c r="N22" s="33">
         <f>SUM(N19:N21)</f>
-        <v>1188207.3</v>
+        <v>1205400</v>
       </c>
       <c r="O22" s="26">
         <f>SUM(O19:O21)</f>
-        <v>1188207.3</v>
+        <v>0</v>
       </c>
       <c r="P22" s="59">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="Q22" s="27"/>
       <c r="R22" s="27"/>
@@ -8736,11 +8733,11 @@
       <c r="D23" s="49"/>
       <c r="E23" s="30">
         <f>SUM(計算結果!X14:X15)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="F23" s="26">
         <f>SUM(計算結果!W14:W15)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="G23" s="46">
         <f t="shared" si="1"/>
@@ -8748,18 +8745,18 @@
       </c>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="K23" s="74"/>
+      <c r="K23" s="78"/>
       <c r="L23" s="48" t="s">
         <v>273</v>
       </c>
       <c r="M23" s="49"/>
       <c r="N23" s="30">
         <f>SUM(計算結果!X14:X15)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="O23" s="26">
         <f>SUM(計算結果!W14:W15)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="P23" s="59">
         <f t="shared" si="2"/>
@@ -8776,41 +8773,41 @@
       <c r="D24" s="51"/>
       <c r="E24" s="33">
         <f>E22-E23</f>
-        <v>1185707.3</v>
+        <v>1205400</v>
       </c>
       <c r="F24" s="26">
         <f>F22-F23</f>
-        <v>1185707.3</v>
+        <v>0</v>
       </c>
       <c r="G24" s="24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="H24" s="27"/>
       <c r="I24" s="27"/>
-      <c r="K24" s="74"/>
+      <c r="K24" s="78"/>
       <c r="L24" s="50" t="s">
         <v>274</v>
       </c>
       <c r="M24" s="51"/>
       <c r="N24" s="33">
         <f>N22-N23</f>
-        <v>1185707.3</v>
+        <v>1205400</v>
       </c>
       <c r="O24" s="26">
         <f>O22-O23</f>
-        <v>1185707.3</v>
+        <v>0</v>
       </c>
       <c r="P24" s="59">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1205400</v>
       </c>
       <c r="Q24" s="27"/>
       <c r="R24" s="27"/>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B25" s="71"/>
-      <c r="C25" s="78" t="s">
+      <c r="C25" s="82" t="s">
         <v>275</v>
       </c>
       <c r="D25" s="45" t="s">
@@ -8821,16 +8818,16 @@
       </c>
       <c r="F25" s="31">
         <f>SUM(計算結果!W21:W22)</f>
-        <v>46200</v>
+        <v>0</v>
       </c>
       <c r="G25" s="46">
         <f t="shared" si="1"/>
-        <v>-46200</v>
+        <v>0</v>
       </c>
       <c r="H25" s="27"/>
       <c r="I25" s="27"/>
-      <c r="K25" s="74"/>
-      <c r="L25" s="80" t="s">
+      <c r="K25" s="78"/>
+      <c r="L25" s="74" t="s">
         <v>275</v>
       </c>
       <c r="M25" s="42" t="s">
@@ -8841,85 +8838,85 @@
       </c>
       <c r="O25" s="56">
         <f>SUM(計算結果!W21:W22)</f>
-        <v>46200</v>
+        <v>0</v>
       </c>
       <c r="P25" s="60">
         <f t="shared" si="2"/>
-        <v>-46200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B26" s="71"/>
-      <c r="C26" s="78"/>
+      <c r="C26" s="82"/>
       <c r="D26" s="28" t="s">
         <v>277</v>
       </c>
       <c r="E26" s="30">
         <v>0</v>
       </c>
-      <c r="F26" s="31">
+      <c r="F26" s="31" t="e">
         <f>SUM(計算結果!W30:W31)</f>
-        <v>237140</v>
-      </c>
-      <c r="G26" s="46">
+        <v>#N/A</v>
+      </c>
+      <c r="G26" s="46" t="e">
         <f t="shared" si="1"/>
-        <v>-237140</v>
+        <v>#N/A</v>
       </c>
       <c r="H26" s="27"/>
       <c r="I26" s="27"/>
-      <c r="K26" s="74"/>
-      <c r="L26" s="81"/>
+      <c r="K26" s="78"/>
+      <c r="L26" s="75"/>
       <c r="M26" s="52" t="s">
         <v>277</v>
       </c>
       <c r="N26">
         <v>0</v>
       </c>
-      <c r="O26" s="63">
+      <c r="O26" s="63" t="e">
         <f>SUM(計算結果!W30:W31)</f>
-        <v>237140</v>
-      </c>
-      <c r="P26" s="62">
+        <v>#N/A</v>
+      </c>
+      <c r="P26" s="62" t="e">
         <f t="shared" si="2"/>
-        <v>-237140</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B27" s="72"/>
-      <c r="C27" s="79"/>
+      <c r="C27" s="83"/>
       <c r="D27" s="47" t="s">
         <v>278</v>
       </c>
       <c r="E27" s="33">
         <v>0</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="26" t="e">
         <f>SUM(F25:F26)</f>
-        <v>283340</v>
-      </c>
-      <c r="G27" s="24">
+        <v>#N/A</v>
+      </c>
+      <c r="G27" s="24" t="e">
         <f t="shared" si="1"/>
-        <v>-283340</v>
+        <v>#N/A</v>
       </c>
       <c r="H27" s="27" t="s">
         <v>279</v>
       </c>
       <c r="I27" s="27"/>
-      <c r="K27" s="74"/>
-      <c r="L27" s="81"/>
+      <c r="K27" s="78"/>
+      <c r="L27" s="75"/>
       <c r="M27" s="53" t="s">
         <v>280</v>
       </c>
       <c r="N27">
         <v>0</v>
       </c>
-      <c r="O27" s="63">
+      <c r="O27" s="63" t="e">
         <f>SUM(計算結果!W33:W34)</f>
-        <v>155662</v>
-      </c>
-      <c r="P27" s="61">
+        <v>#N/A</v>
+      </c>
+      <c r="P27" s="61" t="e">
         <f t="shared" si="2"/>
-        <v>-155662</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.45">
@@ -8928,21 +8925,21 @@
       <c r="G28" s="27"/>
       <c r="H28" s="27"/>
       <c r="I28" s="27"/>
-      <c r="K28" s="75"/>
-      <c r="L28" s="82"/>
+      <c r="K28" s="79"/>
+      <c r="L28" s="76"/>
       <c r="M28" s="47" t="s">
         <v>278</v>
       </c>
       <c r="N28" s="54">
         <v>0</v>
       </c>
-      <c r="O28" s="59">
+      <c r="O28" s="59" t="e">
         <f>SUM(O25:O27)</f>
-        <v>439002</v>
-      </c>
-      <c r="P28" s="59">
+        <v>#N/A</v>
+      </c>
+      <c r="P28" s="59" t="e">
         <f t="shared" si="2"/>
-        <v>-439002</v>
+        <v>#N/A</v>
       </c>
       <c r="Q28" t="s">
         <v>279</v>
@@ -8954,15 +8951,15 @@
       </c>
       <c r="E29" s="55">
         <f>E13+E22-E27</f>
-        <v>3572814.0599999996</v>
-      </c>
-      <c r="F29" s="55">
+        <v>1205400</v>
+      </c>
+      <c r="F29" s="55" t="e">
         <f>F13+F22-F27</f>
-        <v>3289474.0599999996</v>
-      </c>
-      <c r="G29" s="26">
+        <v>#N/A</v>
+      </c>
+      <c r="G29" s="26" t="e">
         <f>E29-F29</f>
-        <v>283340</v>
+        <v>#N/A</v>
       </c>
       <c r="H29" s="27" t="s">
         <v>282</v>
@@ -8980,15 +8977,15 @@
       </c>
       <c r="N30" s="55">
         <f>N13+N22-N28</f>
-        <v>3572814.0599999996</v>
-      </c>
-      <c r="O30" s="55">
+        <v>1205400</v>
+      </c>
+      <c r="O30" s="55" t="e">
         <f>O13+O22-O28</f>
-        <v>3133812.0599999996</v>
-      </c>
-      <c r="P30" s="26">
+        <v>#N/A</v>
+      </c>
+      <c r="P30" s="26" t="e">
         <f>N30-O30</f>
-        <v>439002</v>
+        <v>#N/A</v>
       </c>
       <c r="Q30" s="27" t="s">
         <v>282</v>
@@ -9004,12 +9001,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B5:B13"/>
-    <mergeCell ref="K5:K13"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="L10:L13"/>
     <mergeCell ref="B15:B27"/>
     <mergeCell ref="K15:K28"/>
     <mergeCell ref="C17:C18"/>
@@ -9018,6 +9009,12 @@
     <mergeCell ref="L19:L22"/>
     <mergeCell ref="C25:C27"/>
     <mergeCell ref="L25:L28"/>
+    <mergeCell ref="B5:B13"/>
+    <mergeCell ref="K5:K13"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="L10:L13"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9809,16 +9806,8 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="24" spans="10:22" x14ac:dyDescent="0.45">
-      <c r="Q24" s="3" t="s">
-        <v>284</v>
-      </c>
-    </row>
     <row r="26" spans="10:22" x14ac:dyDescent="0.45">
-      <c r="Q26" s="64" cm="1">
-        <f t="array" ref="Q26">INDEX(マスター!$AA$4:$AA$8,MATCH(1,(計算結果!$AA$49&gt;=マスター!$X$4:$X$8)*(計算結果!$AA$49&lt;=IF(マスター!$Z$4:$Z$8="",1E+99,マスター!$Z$4:$Z$8)),0))</f>
-        <v>0.59838030795460595</v>
-      </c>
+      <c r="Q26" s="64"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -9850,7 +9839,7 @@
       </c>
       <c r="B2" s="3">
         <f>計算結果!W7</f>
-        <v>11882000</v>
+        <v>0</v>
       </c>
       <c r="C2"/>
     </row>
@@ -9860,7 +9849,7 @@
       </c>
       <c r="B3" s="3">
         <f>計算結果!W17+計算結果!W18</f>
-        <v>1185700</v>
+        <v>0</v>
       </c>
       <c r="C3"/>
     </row>
@@ -9876,7 +9865,7 @@
   _xlpm.factor, マスター!$V$3:$V$9+0,
   _xlfn.XLOOKUP(_xlpm.x, _xlpm.lower, _xlpm.factor, , 1)
 )</f>
-        <v>0.56306999999999996</v>
+        <v>0.84894999999999998</v>
       </c>
       <c r="C4"/>
     </row>
@@ -9905,7 +9894,7 @@
       <c r="A8" t="s">
         <v>218</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="3" t="e">
         <f xml:space="preserve">
 ROUNDDOWN(
   ( (計算結果!$W$17 + 計算結果!$W$18) * 0.2 ) /
@@ -9913,7 +9902,7 @@
   + 2000,
   0
 )</f>
-        <v>423155</v>
+        <v>#N/A</v>
       </c>
       <c r="C8"/>
     </row>
@@ -9921,7 +9910,7 @@
       <c r="A9" t="s">
         <v>220</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="16" t="e">
         <f xml:space="preserve">
 ROUNDDOWN(
   ( (計算結果!$W$17 + 計算結果!$W$18) * 0.2 ) /
@@ -9929,7 +9918,7 @@
   + 2000,
   0
 )</f>
-        <v>423155</v>
+        <v>#N/A</v>
       </c>
       <c r="C9"/>
     </row>
@@ -9981,9 +9970,9 @@
       <c r="A16" t="s">
         <v>225</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="3" t="e">
         <f>MIN($B$8,$B$12,$B$13)</f>
-        <v>423155</v>
+        <v>#N/A</v>
       </c>
       <c r="C16"/>
     </row>
@@ -9991,9 +9980,9 @@
       <c r="A17" t="s">
         <v>226</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="3" t="e">
         <f>MIN($B$9,$B$13)</f>
-        <v>423155</v>
+        <v>#N/A</v>
       </c>
       <c r="C17"/>
     </row>

</xml_diff>